<commit_message>
Optimize hashing and add new evaluations
</commit_message>
<xml_diff>
--- a/straight_redis_client/profiling/redis_client_profiling.xlsx
+++ b/straight_redis_client/profiling/redis_client_profiling.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\straight_redis_client\profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7929C4AC-9FE9-49CA-88D4-482E78CC2442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F79BF4-3682-4055-AE6D-91518952F628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ping" sheetId="1" r:id="rId1"/>
-    <sheet name="set" sheetId="9" r:id="rId2"/>
-    <sheet name="get" sheetId="3" r:id="rId3"/>
-    <sheet name="get_range" sheetId="4" r:id="rId4"/>
-    <sheet name="delete" sheetId="5" r:id="rId5"/>
+    <sheet name="Ping Message" sheetId="1" r:id="rId1"/>
+    <sheet name="Set Function" sheetId="9" r:id="rId2"/>
+    <sheet name="Get Function" sheetId="3" r:id="rId3"/>
+    <sheet name="Get-Range Function" sheetId="4" r:id="rId4"/>
+    <sheet name="Delete Function" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -33,9 +33,6 @@
   </si>
   <si>
     <t>Client_Instances=1</t>
-  </si>
-  <si>
-    <t>Wall_Time(seconds)</t>
   </si>
   <si>
     <t>Wall Time: Time taken from sending the response and receiving the response back</t>
@@ -74,9 +71,6 @@
     <t>Redis_DB=10.0.2.82:6379</t>
   </si>
   <si>
-    <t>Wall_Time_Optimized(seconds)</t>
-  </si>
-  <si>
     <t>Optimized with pipeline operators</t>
   </si>
   <si>
@@ -84,6 +78,12 @@
   </si>
   <si>
     <t>Throughput(Number_of_Key_Value_Pairs)</t>
+  </si>
+  <si>
+    <t>Response_Time (seconds)</t>
+  </si>
+  <si>
+    <t>Response_Time_Optimized (seconds)</t>
   </si>
 </sst>
 </file>
@@ -582,13 +582,13 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -601,10 +601,10 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>3</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="12"/>
@@ -702,7 +702,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -747,12 +747,12 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="5"/>
     </row>
@@ -979,13 +979,13 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -998,21 +998,21 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -1026,7 +1026,7 @@
         <v>2.9214599984697998E-3</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -1040,7 +1040,7 @@
         <v>2.9676700010895698E-3</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -1054,7 +1054,7 @@
         <v>4.7610499896109104E-3</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
@@ -1071,7 +1071,7 @@
         <v>2.6601759984623601E-2</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H10" s="7"/>
     </row>
@@ -1124,7 +1124,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1169,12 +1169,12 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="5"/>
     </row>
@@ -1401,13 +1401,13 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -1420,21 +1420,21 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -1448,7 +1448,7 @@
         <v>2.4343300028704098E-3</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -1462,7 +1462,7 @@
         <v>2.5533499894663599E-3</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -1476,7 +1476,7 @@
         <v>5.1798400003463E-3</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
@@ -1493,7 +1493,7 @@
         <v>2.3080520005896599E-2</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H10" s="7"/>
     </row>
@@ -1546,7 +1546,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1591,12 +1591,12 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="5"/>
     </row>
@@ -1822,13 +1822,13 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -1841,21 +1841,21 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -1869,7 +1869,7 @@
         <v>2.9287799960002301E-3</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -1883,7 +1883,7 @@
         <v>3.8782599964178998E-3</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -1897,7 +1897,7 @@
         <v>5.8791999937966403E-3</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
@@ -1914,7 +1914,7 @@
         <v>2.5481500010937401E-2</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H10" s="7"/>
     </row>
@@ -1967,7 +1967,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -2012,12 +2012,12 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="5"/>
     </row>
@@ -2243,13 +2243,13 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -2262,21 +2262,21 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -2290,7 +2290,7 @@
         <v>2.2126199910417199E-3</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -2304,7 +2304,7 @@
         <v>6.3647500122897297E-3</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -2318,7 +2318,7 @@
         <v>9.5526600140146897E-3</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
@@ -2335,7 +2335,7 @@
         <v>1.7872149986214898E-2</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H10" s="7"/>
     </row>
@@ -2388,7 +2388,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -2433,12 +2433,12 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="5"/>
     </row>

</xml_diff>

<commit_message>
Update report profiling and change configs M4
</commit_message>
<xml_diff>
--- a/straight_redis_client/profiling/redis_client_profiling.xlsx
+++ b/straight_redis_client/profiling/redis_client_profiling.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\straight_redis_client\profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1723247-6E52-4C7D-A742-B21470BC924F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382E39CB-F9D9-4377-B927-1AC79CBE8B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ping Message" sheetId="1" r:id="rId1"/>

</xml_diff>